<commit_message>
Registre des écarts : corrections et ajout de l'écart budgétaire E6
- E1 : le cadrage du besoin ayant eu lieu en amont de S1, l'écart porte
  sur les validations intermédiaires, non sur le recueil du besoin
- E2 : arbitrage par la tutrice et non par l'expert métier, indisponible
  sur le sprint 1 ; scénarios validés par le métier à la revue de S2
- E3 : replacé au sprint 1 (05/04 - 24/04/2026), conformément à l'annexe 10
- E6 : réintégration de la ressource prestataire dans le coût complet,
  tracée comme décision de pilotage
- Distinction entre impact sur la dépense et impact sur le périmètre,
  pour lever la contradiction apparente entre budget tenu et périmètre élargi

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TDB_Pilotage_financier_CircuitCle.xlsx
+++ b/TDB_Pilotage_financier_CircuitCle.xlsx
@@ -2235,18 +2235,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="52" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="58" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="58" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2272,31 +2273,36 @@
       </c>
       <c r="E1" s="2" t="inlineStr">
         <is>
-          <t>Impact coût (€)</t>
+          <t>Impact dépense (€)</t>
         </is>
       </c>
       <c r="F1" s="2" t="inlineStr">
         <is>
+          <t>Impact périmètre (€)</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
           <t>Impact délai (j)</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>Décision d'ajustement</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>Arbitré par</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="J1" s="2" t="inlineStr">
         <is>
           <t>Statut</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="46" customHeight="1">
+    <row r="2" ht="52" customHeight="1">
       <c r="A2" s="5" t="inlineStr">
         <is>
           <t>E1</t>
@@ -2314,7 +2320,7 @@
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>Indisponibilité de l'expert métier (Cédric S.) sur l'intégralité du sprint 1</t>
+          <t>Indisponibilité de l'expert métier (Cédric S.) pendant le sprint 1, le cadrage initial du besoin ayant été réalisé en amont du sprint</t>
         </is>
       </c>
       <c r="E2" s="5" t="n">
@@ -2323,23 +2329,26 @@
       <c r="F2" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="G2" s="5" t="inlineStr">
-        <is>
-          <t>Recueil du besoin basculé en asynchrone : tickets Jira et relais de Jonas sur Teams ; revue mensuelle avec le métier instaurée dès S2</t>
-        </is>
+      <c r="G2" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="H2" s="5" t="inlineStr">
         <is>
+          <t>Validations intermédiaires et arbitrages traités en asynchrone (tickets Jira, relais de Jonas sur Teams) ; revue mensuelle avec le métier instaurée dès S2</t>
+        </is>
+      </c>
+      <c r="I2" s="5" t="inlineStr">
+        <is>
           <t>Léna / Jonas</t>
         </is>
       </c>
-      <c r="I2" s="5" t="inlineStr">
+      <c r="J2" s="5" t="inlineStr">
         <is>
           <t>Résolu</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="46" customHeight="1">
+    <row r="3" ht="52" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
         <is>
           <t>E2</t>
@@ -2366,23 +2375,26 @@
       <c r="F3" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="G3" s="5" t="inlineStr">
-        <is>
-          <t>Élargissement du périmètre : génération de 200 logs synthétiques à partir de 6 scénarios REX documentés, portant le dataset à 209 observations</t>
-        </is>
+      <c r="G3" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="H3" s="5" t="inlineStr">
         <is>
-          <t>Léna / Cédric S.</t>
+          <t>Élargissement du périmètre : génération de 200 logs synthétiques à partir de 6 scénarios REX documentés avec le tuteur, portant le dataset à 209 observations ; scénarios validés par le métier à la revue de S2</t>
         </is>
       </c>
       <c r="I3" s="5" t="inlineStr">
         <is>
+          <t>Léna / Jonas</t>
+        </is>
+      </c>
+      <c r="J3" s="5" t="inlineStr">
+        <is>
           <t>Résolu</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="46" customHeight="1">
+    <row r="4" ht="52" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
         <is>
           <t>E3</t>
@@ -2390,7 +2402,7 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>S2</t>
+          <t>S1</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
@@ -2400,7 +2412,7 @@
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>Le découpage aléatoire 70/30 plaçait les cas dangereux dans le jeu de test : accuracy 0,75 et aucune détection de danger</t>
+          <t>Le découpage aléatoire 70/30 plaçait les cas dangereux dans le jeu de test (05/04 – 24/04/2026) : accuracy 0,75 et aucune détection de danger</t>
         </is>
       </c>
       <c r="E4" s="5" t="n">
@@ -2409,23 +2421,26 @@
       <c r="F4" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="G4" s="5" t="inlineStr">
+      <c r="G4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>Révision de la stratégie de séparation : tous les cas dangereux garantis en entraînement, découpage 70/30 appliqué aux seuls cas normaux</t>
         </is>
       </c>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="I4" s="5" t="inlineStr">
         <is>
           <t>Léna</t>
         </is>
       </c>
-      <c r="I4" s="5" t="inlineStr">
+      <c r="J4" s="5" t="inlineStr">
         <is>
           <t>Résolu</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="46" customHeight="1">
+    <row r="5" ht="52" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
           <t>E4</t>
@@ -2452,23 +2467,26 @@
       <c r="F5" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="G5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>Ajustement du périmètre technique : recherche TF-IDF (scikit-learn) retenue à la place des embeddings — exigence ET4 du cahier des charges</t>
         </is>
       </c>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="I5" s="5" t="inlineStr">
         <is>
           <t>Léna / Marius</t>
         </is>
       </c>
-      <c r="I5" s="5" t="inlineStr">
+      <c r="J5" s="5" t="inlineStr">
         <is>
           <t>Résolu</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="46" customHeight="1">
+    <row r="6" ht="52" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
           <t>E5</t>
@@ -2495,19 +2513,68 @@
       <c r="F6" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="G6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>Marge absorbée par le sprint 2, calendrier global maintenu</t>
         </is>
       </c>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="I6" s="5" t="inlineStr">
         <is>
           <t>Léna</t>
         </is>
       </c>
-      <c r="I6" s="5" t="inlineStr">
+      <c r="J6" s="5" t="inlineStr">
         <is>
           <t>Clos</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="52" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>E6</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Bilan</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Périmètre — budget</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Ressource prestataire mutualisée non comptabilisée dans le budget de la première session : le coût affiché ne reflétait pas le coût complet du projet</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="5" t="n">
+        <v>4200</v>
+      </c>
+      <c r="G7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>Réintégration de la quote-part de 25 % du contrat prestataire dans le coût complet (3 751 € → 7 951 €) ; seuil de rentabilité recalculé de 171 à 362 analyses. Aucune dépense supplémentaire : il s'agit d'un élargissement de périmètre, pas d'un dépassement</t>
+        </is>
+      </c>
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>Léna / Jonas</t>
+        </is>
+      </c>
+      <c r="J7" s="5" t="inlineStr">
+        <is>
+          <t>Résolu</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Cadence d'utilisation portée à 25 analyses par mois
Estimation fournie par le métier (Cédric S.) en remplacement de
l'hypothèse de travail à 15. Le délai d'amortissement passe de
24,1 à 14,5 mois.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TDB_Pilotage_financier_CircuitCle.xlsx
+++ b/TDB_Pilotage_financier_CircuitCle.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A37"/>
+  <dimension ref="A1:A38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -685,6 +685,13 @@
       <c r="A37" t="inlineStr">
         <is>
           <t>Curseur de quote-part à 0 % : le tableau de bord retrouve exactement le budget de la thèse (3 751 €, 171 analyses).</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Cadence d'utilisation : 25 analyses par mois, estimation du métier (Cédric S.) — amortissement en 14,5 mois.</t>
         </is>
       </c>
     </row>
@@ -937,7 +944,7 @@
         </is>
       </c>
       <c r="B12" s="3" t="n">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -946,7 +953,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Paramètre de simulation — cadence à caler avec le métier</t>
+          <t>Estimation du métier (Cédric S.)</t>
         </is>
       </c>
     </row>

</xml_diff>